<commit_message>
#28 eSpark BOM update
</commit_message>
<xml_diff>
--- a/Design Files/BLDC-Board-v1.0/BOM/eSpark_BOM_BLDC-Board-v1.0.xlsx
+++ b/Design Files/BLDC-Board-v1.0/BOM/eSpark_BOM_BLDC-Board-v1.0.xlsx
@@ -12,14 +12,14 @@
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="415">
   <si>
     <t>Component list</t>
   </si>
@@ -978,9 +978,6 @@
     <t>C706876</t>
   </si>
   <si>
-    <t>C168677</t>
-  </si>
-  <si>
     <t>C706880</t>
   </si>
   <si>
@@ -1258,6 +1255,15 @@
   </si>
   <si>
     <t>C96446</t>
+  </si>
+  <si>
+    <t>2.54-1*3P</t>
+  </si>
+  <si>
+    <t>C49257</t>
+  </si>
+  <si>
+    <t>C2688120</t>
   </si>
 </sst>
 </file>
@@ -1461,7 +1467,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -1587,21 +1593,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1706,24 +1703,10 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1743,6 +1726,17 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2068,14 +2062,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="42"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="50"/>
+      <c r="N1" s="50"/>
+      <c r="O1" s="50"/>
+      <c r="P1" s="50"/>
+      <c r="Q1" s="50"/>
+      <c r="R1" s="50"/>
     </row>
     <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2086,7 +2080,7 @@
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="40" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="G2" s="5"/>
       <c r="H2" s="3"/>
@@ -2110,7 +2104,7 @@
       </c>
       <c r="E3" s="27"/>
       <c r="F3" s="41" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="G3" s="29"/>
       <c r="H3" s="30"/>
@@ -2209,34 +2203,34 @@
         <v>263</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="J7" s="12" t="s">
         <v>297</v>
       </c>
       <c r="K7" s="12" t="s">
+        <v>396</v>
+      </c>
+      <c r="L7" s="12" t="s">
+        <v>392</v>
+      </c>
+      <c r="M7" s="12" t="s">
         <v>397</v>
       </c>
-      <c r="L7" s="12" t="s">
-        <v>393</v>
-      </c>
-      <c r="M7" s="12" t="s">
+      <c r="N7" s="12" t="s">
         <v>398</v>
       </c>
-      <c r="N7" s="12" t="s">
+      <c r="O7" s="12" t="s">
         <v>399</v>
       </c>
-      <c r="O7" s="12" t="s">
+      <c r="P7" s="12" t="s">
         <v>400</v>
       </c>
-      <c r="P7" s="12" t="s">
+      <c r="Q7" s="12" t="s">
         <v>401</v>
       </c>
-      <c r="Q7" s="12" t="s">
+      <c r="R7" s="12" t="s">
         <v>402</v>
-      </c>
-      <c r="R7" s="12" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
@@ -2263,12 +2257,14 @@
       <c r="H8" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I8" s="14"/>
+      <c r="I8" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J8" s="14" t="s">
         <v>298</v>
       </c>
       <c r="K8" s="14" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="L8" s="14">
         <v>4</v>
@@ -2280,8 +2276,8 @@
       <c r="N8" s="14">
         <v>100</v>
       </c>
-      <c r="O8" s="52" t="s">
-        <v>410</v>
+      <c r="O8" s="48" t="s">
+        <v>409</v>
       </c>
       <c r="P8" s="15">
         <v>1.6000000000000001E-3</v>
@@ -2316,12 +2312,14 @@
       <c r="H9" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I9" s="20"/>
+      <c r="I9" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J9" s="20" t="s">
         <v>299</v>
       </c>
       <c r="K9" s="20" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="L9" s="20">
         <v>1</v>
@@ -2333,8 +2331,8 @@
       <c r="N9" s="20">
         <v>20</v>
       </c>
-      <c r="O9" s="53" t="s">
-        <v>410</v>
+      <c r="O9" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P9" s="21">
         <v>2.0799999999999999E-2</v>
@@ -2354,49 +2352,51 @@
       <c r="C10" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="D10" s="49" t="s">
+      <c r="D10" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="49" t="s">
+      <c r="E10" s="45" t="s">
         <v>102</v>
       </c>
-      <c r="F10" s="48" t="s">
+      <c r="F10" s="44" t="s">
         <v>167</v>
       </c>
-      <c r="G10" s="49" t="s">
+      <c r="G10" s="45" t="s">
         <v>206</v>
       </c>
-      <c r="H10" s="49" t="s">
+      <c r="H10" s="45" t="s">
         <v>264</v>
       </c>
-      <c r="I10" s="49"/>
-      <c r="J10" s="49" t="s">
+      <c r="I10" s="14" t="s">
+        <v>310</v>
+      </c>
+      <c r="J10" s="45" t="s">
         <v>300</v>
       </c>
-      <c r="K10" s="49" t="s">
-        <v>362</v>
-      </c>
-      <c r="L10" s="49">
+      <c r="K10" s="45" t="s">
+        <v>361</v>
+      </c>
+      <c r="L10" s="45">
         <v>2</v>
       </c>
-      <c r="M10" s="49">
+      <c r="M10" s="45">
         <f>L10*5</f>
         <v>10</v>
       </c>
-      <c r="N10" s="45" t="s">
-        <v>310</v>
-      </c>
-      <c r="O10" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P10" s="50" t="s">
-        <v>310</v>
-      </c>
-      <c r="Q10" s="50" t="s">
-        <v>310</v>
-      </c>
-      <c r="R10" s="51" t="s">
-        <v>405</v>
+      <c r="N10" s="42" t="s">
+        <v>310</v>
+      </c>
+      <c r="O10" s="43" t="s">
+        <v>409</v>
+      </c>
+      <c r="P10" s="46" t="s">
+        <v>310</v>
+      </c>
+      <c r="Q10" s="46" t="s">
+        <v>310</v>
+      </c>
+      <c r="R10" s="47" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
@@ -2423,12 +2423,14 @@
       <c r="H11" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="I11" s="20"/>
+      <c r="I11" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J11" s="20" t="s">
         <v>301</v>
       </c>
       <c r="K11" s="20" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="L11" s="20">
         <v>2</v>
@@ -2440,8 +2442,8 @@
       <c r="N11" s="20">
         <v>100</v>
       </c>
-      <c r="O11" s="53" t="s">
-        <v>410</v>
+      <c r="O11" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P11" s="21">
         <v>2.0999999999999999E-3</v>
@@ -2476,12 +2478,14 @@
       <c r="H12" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I12" s="14"/>
+      <c r="I12" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J12" s="14" t="s">
         <v>302</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="L12" s="14">
         <v>1</v>
@@ -2493,8 +2497,8 @@
       <c r="N12" s="14">
         <v>50</v>
       </c>
-      <c r="O12" s="53" t="s">
-        <v>410</v>
+      <c r="O12" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P12" s="15">
         <v>1.7500000000000002E-2</v>
@@ -2529,12 +2533,14 @@
       <c r="H13" s="20" t="s">
         <v>266</v>
       </c>
-      <c r="I13" s="20"/>
+      <c r="I13" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J13" s="20" t="s">
         <v>303</v>
       </c>
       <c r="K13" s="20" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="L13" s="20">
         <v>6</v>
@@ -2546,8 +2552,8 @@
       <c r="N13" s="20">
         <v>40</v>
       </c>
-      <c r="O13" s="53" t="s">
-        <v>410</v>
+      <c r="O13" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P13" s="21">
         <v>1.32E-2</v>
@@ -2582,12 +2588,14 @@
       <c r="H14" s="14" t="s">
         <v>266</v>
       </c>
-      <c r="I14" s="14"/>
+      <c r="I14" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J14" s="14" t="s">
         <v>304</v>
       </c>
       <c r="K14" s="14" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="L14" s="14">
         <v>1</v>
@@ -2599,8 +2607,8 @@
       <c r="N14" s="14">
         <v>10</v>
       </c>
-      <c r="O14" s="53" t="s">
-        <v>410</v>
+      <c r="O14" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P14" s="15">
         <v>9.4500000000000001E-2</v>
@@ -2635,12 +2643,14 @@
       <c r="H15" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="I15" s="20"/>
+      <c r="I15" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J15" s="20" t="s">
         <v>305</v>
       </c>
       <c r="K15" s="20" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="L15" s="20">
         <v>1</v>
@@ -2652,8 +2662,8 @@
       <c r="N15" s="20">
         <v>20</v>
       </c>
-      <c r="O15" s="53" t="s">
-        <v>410</v>
+      <c r="O15" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P15" s="21">
         <v>2.1100000000000001E-2</v>
@@ -2682,20 +2692,20 @@
       <c r="F16" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="G16" s="45" t="s">
+      <c r="G16" s="42" t="s">
         <v>212</v>
       </c>
       <c r="H16" s="14" t="s">
         <v>266</v>
       </c>
       <c r="I16" s="14" t="s">
+        <v>410</v>
+      </c>
+      <c r="J16" s="14" t="s">
         <v>411</v>
       </c>
-      <c r="J16" s="14" t="s">
-        <v>412</v>
-      </c>
       <c r="K16" s="14" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="L16" s="14">
         <v>3</v>
@@ -2707,8 +2717,8 @@
       <c r="N16" s="14">
         <v>50</v>
       </c>
-      <c r="O16" s="53" t="s">
-        <v>410</v>
+      <c r="O16" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P16" s="15">
         <v>1.67E-2</v>
@@ -2735,7 +2745,7 @@
         <v>109</v>
       </c>
       <c r="F17" s="20" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G17" s="20" t="s">
         <v>170</v>
@@ -2743,12 +2753,14 @@
       <c r="H17" s="20" t="s">
         <v>267</v>
       </c>
-      <c r="I17" s="20"/>
+      <c r="I17" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J17" s="20" t="s">
         <v>306</v>
       </c>
       <c r="K17" s="20" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="L17" s="20">
         <v>6</v>
@@ -2760,8 +2772,8 @@
       <c r="N17" s="20">
         <v>31</v>
       </c>
-      <c r="O17" s="53" t="s">
-        <v>410</v>
+      <c r="O17" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P17" s="21">
         <v>0.16900000000000001</v>
@@ -2796,12 +2808,14 @@
       <c r="H18" s="14" t="s">
         <v>268</v>
       </c>
-      <c r="I18" s="14"/>
+      <c r="I18" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J18" s="14" t="s">
         <v>307</v>
       </c>
       <c r="K18" s="14" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="L18" s="14">
         <v>3</v>
@@ -2813,8 +2827,8 @@
       <c r="N18" s="14">
         <v>20</v>
       </c>
-      <c r="O18" s="53" t="s">
-        <v>410</v>
+      <c r="O18" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P18" s="15">
         <v>0.29310000000000003</v>
@@ -2849,12 +2863,14 @@
       <c r="H19" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I19" s="20"/>
+      <c r="I19" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J19" s="20" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="K19" s="20" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="L19" s="20">
         <v>1</v>
@@ -2866,8 +2882,8 @@
       <c r="N19" s="20">
         <v>100</v>
       </c>
-      <c r="O19" s="53" t="s">
-        <v>410</v>
+      <c r="O19" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P19" s="21">
         <v>1E-3</v>
@@ -2902,12 +2918,14 @@
       <c r="H20" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="I20" s="14"/>
+      <c r="I20" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J20" s="14" t="s">
         <v>308</v>
       </c>
       <c r="K20" s="14" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="L20" s="14">
         <v>6</v>
@@ -2919,8 +2937,8 @@
       <c r="N20" s="14">
         <v>50</v>
       </c>
-      <c r="O20" s="53" t="s">
-        <v>410</v>
+      <c r="O20" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P20" s="15">
         <v>8.3999999999999995E-3</v>
@@ -2955,7 +2973,9 @@
       <c r="H21" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="I21" s="20"/>
+      <c r="I21" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J21" s="20" t="s">
         <v>309</v>
       </c>
@@ -2972,8 +2992,8 @@
       <c r="N21" s="20">
         <v>15</v>
       </c>
-      <c r="O21" s="53" t="s">
-        <v>410</v>
+      <c r="O21" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P21" s="21">
         <v>0.10249999999999999</v>
@@ -3002,15 +3022,17 @@
       <c r="F22" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="G22" s="14" t="s">
+      <c r="G22" s="42" t="s">
         <v>217</v>
       </c>
       <c r="H22" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="I22" s="14"/>
+      <c r="I22" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J22" s="14" t="s">
-        <v>310</v>
+        <v>414</v>
       </c>
       <c r="K22" s="20" t="s">
         <v>310</v>
@@ -3022,14 +3044,18 @@
         <f>L22*5</f>
         <v>10</v>
       </c>
-      <c r="N22" s="14"/>
-      <c r="O22" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P22" s="15"/>
+      <c r="N22" s="14">
+        <v>20</v>
+      </c>
+      <c r="O22" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P22" s="15">
+        <v>3.3500000000000002E-2</v>
+      </c>
       <c r="Q22" s="15">
         <f>P22*N22</f>
-        <v>0</v>
+        <v>0.67</v>
       </c>
       <c r="R22" s="14"/>
     </row>
@@ -3057,9 +3083,11 @@
       <c r="H23" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="I23" s="20"/>
+      <c r="I23" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J23" s="20" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="K23" s="20" t="s">
         <v>310</v>
@@ -3074,8 +3102,8 @@
       <c r="N23" s="20">
         <v>10</v>
       </c>
-      <c r="O23" s="53" t="s">
-        <v>410</v>
+      <c r="O23" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P23" s="21">
         <v>0.153</v>
@@ -3110,7 +3138,9 @@
       <c r="H24" s="14" t="s">
         <v>272</v>
       </c>
-      <c r="I24" s="14"/>
+      <c r="I24" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J24" s="14" t="s">
         <v>311</v>
       </c>
@@ -3127,8 +3157,8 @@
       <c r="N24" s="14">
         <v>20</v>
       </c>
-      <c r="O24" s="53" t="s">
-        <v>410</v>
+      <c r="O24" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P24" s="15">
         <v>3.0800000000000001E-2</v>
@@ -3163,7 +3193,9 @@
       <c r="H25" s="20" t="s">
         <v>273</v>
       </c>
-      <c r="I25" s="20"/>
+      <c r="I25" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J25" s="20" t="s">
         <v>312</v>
       </c>
@@ -3180,8 +3212,8 @@
       <c r="N25" s="20">
         <v>30</v>
       </c>
-      <c r="O25" s="53" t="s">
-        <v>410</v>
+      <c r="O25" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P25" s="21">
         <v>2.6700000000000002E-2</v>
@@ -3216,7 +3248,9 @@
       <c r="H26" s="14" t="s">
         <v>271</v>
       </c>
-      <c r="I26" s="14"/>
+      <c r="I26" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J26" s="14" t="s">
         <v>313</v>
       </c>
@@ -3233,8 +3267,8 @@
       <c r="N26" s="14">
         <v>50</v>
       </c>
-      <c r="O26" s="53" t="s">
-        <v>410</v>
+      <c r="O26" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P26" s="15">
         <v>1.29E-2</v>
@@ -3269,7 +3303,9 @@
       <c r="H27" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="I27" s="20"/>
+      <c r="I27" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J27" s="20" t="s">
         <v>314</v>
       </c>
@@ -3286,8 +3322,8 @@
       <c r="N27" s="20">
         <v>50</v>
       </c>
-      <c r="O27" s="53" t="s">
-        <v>410</v>
+      <c r="O27" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P27" s="21">
         <v>1.29E-2</v>
@@ -3322,7 +3358,9 @@
       <c r="H28" s="14" t="s">
         <v>269</v>
       </c>
-      <c r="I28" s="14"/>
+      <c r="I28" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J28" s="14" t="s">
         <v>315</v>
       </c>
@@ -3339,8 +3377,8 @@
       <c r="N28" s="14">
         <v>50</v>
       </c>
-      <c r="O28" s="53" t="s">
-        <v>410</v>
+      <c r="O28" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P28" s="15">
         <v>4.5999999999999999E-2</v>
@@ -3375,7 +3413,9 @@
       <c r="H29" s="20" t="s">
         <v>275</v>
       </c>
-      <c r="I29" s="20"/>
+      <c r="I29" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J29" s="20" t="s">
         <v>316</v>
       </c>
@@ -3392,8 +3432,8 @@
       <c r="N29" s="20">
         <v>30</v>
       </c>
-      <c r="O29" s="53" t="s">
-        <v>410</v>
+      <c r="O29" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P29" s="21">
         <v>5.45E-2</v>
@@ -3420,7 +3460,7 @@
         <v>122</v>
       </c>
       <c r="F30" s="20" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G30" s="14" t="s">
         <v>225</v>
@@ -3428,7 +3468,9 @@
       <c r="H30" s="14" t="s">
         <v>276</v>
       </c>
-      <c r="I30" s="14"/>
+      <c r="I30" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J30" s="14" t="s">
         <v>317</v>
       </c>
@@ -3445,8 +3487,8 @@
       <c r="N30" s="14">
         <v>10</v>
       </c>
-      <c r="O30" s="53" t="s">
-        <v>410</v>
+      <c r="O30" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P30" s="15">
         <v>0.1482</v>
@@ -3481,7 +3523,9 @@
       <c r="H31" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="I31" s="20"/>
+      <c r="I31" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J31" s="20" t="s">
         <v>318</v>
       </c>
@@ -3498,8 +3542,8 @@
       <c r="N31" s="20">
         <v>20</v>
       </c>
-      <c r="O31" s="53" t="s">
-        <v>410</v>
+      <c r="O31" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P31" s="21">
         <v>5.1299999999999998E-2</v>
@@ -3528,15 +3572,17 @@
       <c r="F32" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="G32" s="47" t="s">
-        <v>371</v>
+      <c r="G32" s="42" t="s">
+        <v>370</v>
       </c>
       <c r="H32" s="14" t="s">
-        <v>406</v>
-      </c>
-      <c r="I32" s="14"/>
+        <v>405</v>
+      </c>
+      <c r="I32" s="20" t="s">
+        <v>412</v>
+      </c>
       <c r="J32" s="14" t="s">
-        <v>319</v>
+        <v>413</v>
       </c>
       <c r="K32" s="20" t="s">
         <v>310</v>
@@ -3548,14 +3594,18 @@
         <f>L32*5</f>
         <v>5</v>
       </c>
-      <c r="N32" s="14"/>
-      <c r="O32" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P32" s="15"/>
+      <c r="N32" s="14">
+        <v>50</v>
+      </c>
+      <c r="O32" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P32" s="15">
+        <v>1.4500000000000001E-2</v>
+      </c>
       <c r="Q32" s="15">
         <f>P32*N32</f>
-        <v>0</v>
+        <v>0.72500000000000009</v>
       </c>
       <c r="R32" s="14"/>
     </row>
@@ -3583,9 +3633,11 @@
       <c r="H33" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="I33" s="20"/>
+      <c r="I33" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J33" s="20" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="K33" s="20" t="s">
         <v>310</v>
@@ -3600,8 +3652,8 @@
       <c r="N33" s="20">
         <v>10</v>
       </c>
-      <c r="O33" s="53" t="s">
-        <v>410</v>
+      <c r="O33" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P33" s="21">
         <v>0.10249999999999999</v>
@@ -3628,7 +3680,7 @@
         <v>126</v>
       </c>
       <c r="F34" s="20" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G34" s="14" t="s">
         <v>183</v>
@@ -3636,9 +3688,11 @@
       <c r="H34" s="14" t="s">
         <v>278</v>
       </c>
-      <c r="I34" s="14"/>
+      <c r="I34" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J34" s="14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="K34" s="20" t="s">
         <v>310</v>
@@ -3653,8 +3707,8 @@
       <c r="N34" s="14">
         <v>25</v>
       </c>
-      <c r="O34" s="53" t="s">
-        <v>410</v>
+      <c r="O34" s="49" t="s">
+        <v>409</v>
       </c>
       <c r="P34" s="15">
         <v>0.26019999999999999</v>
@@ -3681,7 +3735,7 @@
         <v>127</v>
       </c>
       <c r="F35" s="20" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G35" s="20" t="s">
         <v>184</v>
@@ -3689,9 +3743,11 @@
       <c r="H35" s="20" t="s">
         <v>278</v>
       </c>
-      <c r="I35" s="20"/>
+      <c r="I35" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J35" s="20" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="K35" s="20" t="s">
         <v>310</v>
@@ -3703,14 +3759,18 @@
         <f t="shared" ref="M35" si="27">L35*5</f>
         <v>5</v>
       </c>
-      <c r="N35" s="20"/>
-      <c r="O35" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P35" s="21"/>
+      <c r="N35" s="20">
+        <v>10</v>
+      </c>
+      <c r="O35" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P35" s="21">
+        <v>0.16550000000000001</v>
+      </c>
       <c r="Q35" s="21">
         <f t="shared" ref="Q35" si="28">P35*N35</f>
-        <v>0</v>
+        <v>1.655</v>
       </c>
       <c r="R35" s="20"/>
     </row>
@@ -3730,7 +3790,7 @@
         <v>128</v>
       </c>
       <c r="F36" s="20" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G36" s="14">
         <v>1715721</v>
@@ -3738,9 +3798,11 @@
       <c r="H36" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="I36" s="14"/>
+      <c r="I36" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J36" s="14" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="K36" s="20" t="s">
         <v>310</v>
@@ -3752,14 +3814,18 @@
         <f>L36*5</f>
         <v>15</v>
       </c>
-      <c r="N36" s="14"/>
-      <c r="O36" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P36" s="15"/>
+      <c r="N36" s="14">
+        <v>16</v>
+      </c>
+      <c r="O36" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P36" s="15">
+        <v>0.30509999999999998</v>
+      </c>
       <c r="Q36" s="15">
         <f>P36*N36</f>
-        <v>0</v>
+        <v>4.8815999999999997</v>
       </c>
       <c r="R36" s="14"/>
     </row>
@@ -3779,7 +3845,7 @@
         <v>129</v>
       </c>
       <c r="F37" s="20" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G37" s="20" t="s">
         <v>185</v>
@@ -3787,9 +3853,11 @@
       <c r="H37" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="I37" s="20"/>
+      <c r="I37" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J37" s="20" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="K37" s="20" t="s">
         <v>310</v>
@@ -3801,14 +3869,18 @@
         <f t="shared" ref="M37" si="29">L37*5</f>
         <v>20</v>
       </c>
-      <c r="N37" s="20"/>
-      <c r="O37" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P37" s="21"/>
+      <c r="N37" s="20">
+        <v>21</v>
+      </c>
+      <c r="O37" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P37" s="21">
+        <v>0.76639999999999997</v>
+      </c>
       <c r="Q37" s="21">
         <f t="shared" ref="Q37" si="30">P37*N37</f>
-        <v>0</v>
+        <v>16.0944</v>
       </c>
       <c r="R37" s="20"/>
     </row>
@@ -3836,9 +3908,11 @@
       <c r="H38" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="I38" s="14"/>
+      <c r="I38" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J38" s="14" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="K38" s="20" t="s">
         <v>310</v>
@@ -3850,14 +3924,18 @@
         <f>L38*5</f>
         <v>5</v>
       </c>
-      <c r="N38" s="14"/>
-      <c r="O38" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P38" s="15"/>
+      <c r="N38" s="14">
+        <v>100</v>
+      </c>
+      <c r="O38" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P38" s="15">
+        <v>3.3E-3</v>
+      </c>
       <c r="Q38" s="15">
         <f>P38*N38</f>
-        <v>0</v>
+        <v>0.33</v>
       </c>
       <c r="R38" s="14"/>
     </row>
@@ -3877,7 +3955,7 @@
         <v>131</v>
       </c>
       <c r="F39" s="20" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G39" s="20" t="s">
         <v>229</v>
@@ -3885,12 +3963,14 @@
       <c r="H39" s="20" t="s">
         <v>281</v>
       </c>
-      <c r="I39" s="20"/>
+      <c r="I39" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J39" s="20" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="K39" s="20" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="L39" s="20">
         <v>1</v>
@@ -3899,14 +3979,18 @@
         <f t="shared" ref="M39" si="31">L39*5</f>
         <v>5</v>
       </c>
-      <c r="N39" s="20"/>
-      <c r="O39" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P39" s="21"/>
+      <c r="N39" s="20">
+        <v>10</v>
+      </c>
+      <c r="O39" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P39" s="21">
+        <v>8.9499999999999996E-2</v>
+      </c>
       <c r="Q39" s="21">
         <f t="shared" ref="Q39" si="32">P39*N39</f>
-        <v>0</v>
+        <v>0.89500000000000002</v>
       </c>
       <c r="R39" s="20"/>
     </row>
@@ -3934,9 +4018,11 @@
       <c r="H40" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="I40" s="14"/>
+      <c r="I40" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J40" s="14" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="K40" s="14" t="s">
         <v>310</v>
@@ -3948,14 +4034,18 @@
         <f>L40*5</f>
         <v>15</v>
       </c>
-      <c r="N40" s="14"/>
-      <c r="O40" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P40" s="15"/>
+      <c r="N40" s="14">
+        <v>20</v>
+      </c>
+      <c r="O40" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P40" s="15">
+        <v>2.2700000000000001E-2</v>
+      </c>
       <c r="Q40" s="15">
         <f>P40*N40</f>
-        <v>0</v>
+        <v>0.45400000000000001</v>
       </c>
       <c r="R40" s="14"/>
     </row>
@@ -3983,9 +4073,11 @@
       <c r="H41" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="I41" s="20"/>
+      <c r="I41" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J41" s="20" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="K41" s="14" t="s">
         <v>310</v>
@@ -3997,14 +4089,18 @@
         <f t="shared" ref="M41" si="33">L41*5</f>
         <v>20</v>
       </c>
-      <c r="N41" s="20"/>
-      <c r="O41" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P41" s="21"/>
+      <c r="N41" s="20">
+        <v>40</v>
+      </c>
+      <c r="O41" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P41" s="21">
+        <v>2.12E-2</v>
+      </c>
       <c r="Q41" s="21">
         <f t="shared" ref="Q41" si="34">P41*N41</f>
-        <v>0</v>
+        <v>0.84799999999999998</v>
       </c>
       <c r="R41" s="20"/>
     </row>
@@ -4032,9 +4128,11 @@
       <c r="H42" s="14" t="s">
         <v>283</v>
       </c>
-      <c r="I42" s="14"/>
+      <c r="I42" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J42" s="14" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="K42" s="14" t="s">
         <v>310</v>
@@ -4046,14 +4144,18 @@
         <f>L42*5</f>
         <v>20</v>
       </c>
-      <c r="N42" s="14"/>
-      <c r="O42" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P42" s="15"/>
+      <c r="N42" s="14">
+        <v>50</v>
+      </c>
+      <c r="O42" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P42" s="15">
+        <v>1.3299999999999999E-2</v>
+      </c>
       <c r="Q42" s="15">
         <f>P42*N42</f>
-        <v>0</v>
+        <v>0.66499999999999992</v>
       </c>
       <c r="R42" s="14"/>
     </row>
@@ -4081,9 +4183,11 @@
       <c r="H43" s="20" t="s">
         <v>284</v>
       </c>
-      <c r="I43" s="20"/>
+      <c r="I43" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J43" s="20" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="K43" s="14" t="s">
         <v>310</v>
@@ -4095,14 +4199,18 @@
         <f t="shared" ref="M43" si="35">L43*5</f>
         <v>20</v>
       </c>
-      <c r="N43" s="20"/>
-      <c r="O43" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P43" s="21"/>
+      <c r="N43" s="20">
+        <v>50</v>
+      </c>
+      <c r="O43" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P43" s="21">
+        <v>1.5800000000000002E-2</v>
+      </c>
       <c r="Q43" s="21">
         <f t="shared" ref="Q43" si="36">P43*N43</f>
-        <v>0</v>
+        <v>0.79</v>
       </c>
       <c r="R43" s="20"/>
     </row>
@@ -4130,12 +4238,14 @@
       <c r="H44" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I44" s="14"/>
+      <c r="I44" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J44" s="14" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="K44" s="14" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="L44" s="14">
         <v>2</v>
@@ -4144,14 +4254,18 @@
         <f>L44*5</f>
         <v>10</v>
       </c>
-      <c r="N44" s="14"/>
-      <c r="O44" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P44" s="15"/>
+      <c r="N44" s="14">
+        <v>100</v>
+      </c>
+      <c r="O44" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P44" s="15">
+        <v>6.9999999999999999E-4</v>
+      </c>
       <c r="Q44" s="15">
         <f>P44*N44</f>
-        <v>0</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="R44" s="14"/>
     </row>
@@ -4179,12 +4293,14 @@
       <c r="H45" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I45" s="20"/>
+      <c r="I45" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J45" s="20" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="K45" s="20" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="L45" s="20">
         <v>1</v>
@@ -4193,14 +4309,18 @@
         <f t="shared" ref="M45" si="37">L45*5</f>
         <v>5</v>
       </c>
-      <c r="N45" s="20"/>
-      <c r="O45" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P45" s="21"/>
+      <c r="N45" s="20">
+        <v>100</v>
+      </c>
+      <c r="O45" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P45" s="21">
+        <v>2.8E-3</v>
+      </c>
       <c r="Q45" s="21">
         <f t="shared" ref="Q45" si="38">P45*N45</f>
-        <v>0</v>
+        <v>0.27999999999999997</v>
       </c>
       <c r="R45" s="20"/>
     </row>
@@ -4213,49 +4333,51 @@
       <c r="C46" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="D46" s="45" t="s">
+      <c r="D46" s="42" t="s">
         <v>69</v>
       </c>
-      <c r="E46" s="45" t="s">
+      <c r="E46" s="42" t="s">
         <v>138</v>
       </c>
-      <c r="F46" s="48" t="s">
+      <c r="F46" s="44" t="s">
         <v>190</v>
       </c>
-      <c r="G46" s="45" t="s">
+      <c r="G46" s="42" t="s">
         <v>236</v>
       </c>
-      <c r="H46" s="45" t="s">
+      <c r="H46" s="42" t="s">
         <v>264</v>
       </c>
-      <c r="I46" s="45"/>
-      <c r="J46" s="45" t="s">
-        <v>332</v>
-      </c>
-      <c r="K46" s="45" t="s">
-        <v>362</v>
-      </c>
-      <c r="L46" s="45">
+      <c r="I46" s="42" t="s">
+        <v>310</v>
+      </c>
+      <c r="J46" s="42" t="s">
+        <v>331</v>
+      </c>
+      <c r="K46" s="42" t="s">
+        <v>361</v>
+      </c>
+      <c r="L46" s="42">
         <v>2</v>
       </c>
-      <c r="M46" s="45">
+      <c r="M46" s="42">
         <f>L46*5</f>
         <v>10</v>
       </c>
-      <c r="N46" s="45" t="s">
-        <v>310</v>
-      </c>
-      <c r="O46" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P46" s="50" t="s">
-        <v>310</v>
-      </c>
-      <c r="Q46" s="50" t="s">
-        <v>310</v>
-      </c>
-      <c r="R46" s="51" t="s">
-        <v>405</v>
+      <c r="N46" s="42" t="s">
+        <v>310</v>
+      </c>
+      <c r="O46" s="43" t="s">
+        <v>409</v>
+      </c>
+      <c r="P46" s="46" t="s">
+        <v>310</v>
+      </c>
+      <c r="Q46" s="46" t="s">
+        <v>310</v>
+      </c>
+      <c r="R46" s="47" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
@@ -4282,12 +4404,14 @@
       <c r="H47" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I47" s="20"/>
+      <c r="I47" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J47" s="20" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="K47" s="20" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="L47" s="20">
         <v>2</v>
@@ -4296,14 +4420,18 @@
         <f t="shared" ref="M47" si="39">L47*5</f>
         <v>10</v>
       </c>
-      <c r="N47" s="20"/>
-      <c r="O47" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P47" s="21"/>
+      <c r="N47" s="20">
+        <v>100</v>
+      </c>
+      <c r="O47" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P47" s="21">
+        <v>1E-3</v>
+      </c>
       <c r="Q47" s="21">
         <f t="shared" ref="Q47" si="40">P47*N47</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="R47" s="20"/>
     </row>
@@ -4331,12 +4459,14 @@
       <c r="H48" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I48" s="14"/>
+      <c r="I48" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J48" s="14" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="K48" s="14" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="L48" s="14">
         <v>14</v>
@@ -4345,14 +4475,18 @@
         <f>L48*5</f>
         <v>70</v>
       </c>
-      <c r="N48" s="14"/>
-      <c r="O48" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P48" s="15"/>
+      <c r="N48" s="14">
+        <v>100</v>
+      </c>
+      <c r="O48" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P48" s="15">
+        <v>5.0000000000000001E-4</v>
+      </c>
       <c r="Q48" s="15">
         <f>P48*N48</f>
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="R48" s="14"/>
     </row>
@@ -4380,12 +4514,14 @@
       <c r="H49" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I49" s="20"/>
+      <c r="I49" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J49" s="20" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="K49" s="20" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="L49" s="20">
         <v>1</v>
@@ -4394,14 +4530,18 @@
         <f t="shared" ref="M49" si="41">L49*5</f>
         <v>5</v>
       </c>
-      <c r="N49" s="20"/>
-      <c r="O49" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P49" s="21"/>
+      <c r="N49" s="20">
+        <v>20</v>
+      </c>
+      <c r="O49" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P49" s="21">
+        <v>2.7400000000000001E-2</v>
+      </c>
       <c r="Q49" s="21">
         <f t="shared" ref="Q49" si="42">P49*N49</f>
-        <v>0</v>
+        <v>0.54800000000000004</v>
       </c>
       <c r="R49" s="20"/>
     </row>
@@ -4429,12 +4569,14 @@
       <c r="H50" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I50" s="14"/>
+      <c r="I50" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J50" s="14" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="K50" s="14" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="L50" s="14">
         <v>1</v>
@@ -4443,14 +4585,18 @@
         <f>L50*5</f>
         <v>5</v>
       </c>
-      <c r="N50" s="14"/>
-      <c r="O50" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P50" s="15"/>
+      <c r="N50" s="14">
+        <v>50</v>
+      </c>
+      <c r="O50" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P50" s="15">
+        <v>1.8200000000000001E-2</v>
+      </c>
       <c r="Q50" s="15">
         <f>P50*N50</f>
-        <v>0</v>
+        <v>0.91</v>
       </c>
       <c r="R50" s="14"/>
     </row>
@@ -4478,12 +4624,14 @@
       <c r="H51" s="20" t="s">
         <v>285</v>
       </c>
-      <c r="I51" s="20"/>
+      <c r="I51" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J51" s="20" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="K51" s="20" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="L51" s="20">
         <v>4</v>
@@ -4492,14 +4640,18 @@
         <f t="shared" ref="M51" si="43">L51*5</f>
         <v>20</v>
       </c>
-      <c r="N51" s="20"/>
-      <c r="O51" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P51" s="21"/>
+      <c r="N51" s="20">
+        <v>25</v>
+      </c>
+      <c r="O51" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P51" s="21">
+        <v>8.5000000000000006E-2</v>
+      </c>
       <c r="Q51" s="21">
         <f t="shared" ref="Q51" si="44">P51*N51</f>
-        <v>0</v>
+        <v>2.125</v>
       </c>
       <c r="R51" s="20"/>
     </row>
@@ -4527,12 +4679,14 @@
       <c r="H52" s="14" t="s">
         <v>286</v>
       </c>
-      <c r="I52" s="14"/>
+      <c r="I52" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J52" s="14" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="K52" s="14" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="L52" s="14">
         <v>16</v>
@@ -4541,14 +4695,18 @@
         <f>L52*5</f>
         <v>80</v>
       </c>
-      <c r="N52" s="14"/>
-      <c r="O52" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P52" s="15"/>
+      <c r="N52" s="14">
+        <v>100</v>
+      </c>
+      <c r="O52" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P52" s="15">
+        <v>2.07E-2</v>
+      </c>
       <c r="Q52" s="15">
         <f>P52*N52</f>
-        <v>0</v>
+        <v>2.0699999999999998</v>
       </c>
       <c r="R52" s="14"/>
     </row>
@@ -4576,12 +4734,14 @@
       <c r="H53" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I53" s="20"/>
+      <c r="I53" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J53" s="20" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="K53" s="20" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="L53" s="20">
         <v>4</v>
@@ -4590,14 +4750,18 @@
         <f t="shared" ref="M53" si="45">L53*5</f>
         <v>20</v>
       </c>
-      <c r="N53" s="20"/>
-      <c r="O53" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P53" s="21"/>
+      <c r="N53" s="20">
+        <v>30</v>
+      </c>
+      <c r="O53" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P53" s="21">
+        <v>5.57E-2</v>
+      </c>
       <c r="Q53" s="21">
         <f t="shared" ref="Q53" si="46">P53*N53</f>
-        <v>0</v>
+        <v>1.671</v>
       </c>
       <c r="R53" s="20"/>
     </row>
@@ -4625,12 +4789,14 @@
       <c r="H54" s="14" t="s">
         <v>287</v>
       </c>
-      <c r="I54" s="14"/>
+      <c r="I54" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J54" s="14" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="K54" s="14" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="L54" s="14">
         <v>1</v>
@@ -4639,14 +4805,18 @@
         <f>L54*5</f>
         <v>5</v>
       </c>
-      <c r="N54" s="14"/>
-      <c r="O54" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P54" s="15"/>
+      <c r="N54" s="14">
+        <v>100</v>
+      </c>
+      <c r="O54" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P54" s="15">
+        <v>6.9999999999999999E-4</v>
+      </c>
       <c r="Q54" s="15">
         <f>P54*N54</f>
-        <v>0</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="R54" s="14"/>
     </row>
@@ -4672,12 +4842,14 @@
         <v>244</v>
       </c>
       <c r="H55" s="20"/>
-      <c r="I55" s="20"/>
+      <c r="I55" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J55" s="20" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="K55" s="20" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="L55" s="20">
         <v>2</v>
@@ -4686,14 +4858,18 @@
         <f t="shared" ref="M55" si="47">L55*5</f>
         <v>10</v>
       </c>
-      <c r="N55" s="20"/>
-      <c r="O55" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P55" s="21"/>
+      <c r="N55" s="20">
+        <v>100</v>
+      </c>
+      <c r="O55" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P55" s="21">
+        <v>5.9999999999999995E-4</v>
+      </c>
       <c r="Q55" s="21">
         <f t="shared" ref="Q55" si="48">P55*N55</f>
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="R55" s="20"/>
     </row>
@@ -4721,12 +4897,14 @@
       <c r="H56" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I56" s="14"/>
+      <c r="I56" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J56" s="14" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="K56" s="14" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="L56" s="14">
         <v>1</v>
@@ -4735,14 +4913,18 @@
         <f>L56*5</f>
         <v>5</v>
       </c>
-      <c r="N56" s="14"/>
-      <c r="O56" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P56" s="15"/>
+      <c r="N56" s="14">
+        <v>100</v>
+      </c>
+      <c r="O56" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P56" s="15">
+        <v>5.9999999999999995E-4</v>
+      </c>
       <c r="Q56" s="15">
         <f>P56*N56</f>
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="R56" s="14"/>
     </row>
@@ -4770,12 +4952,14 @@
       <c r="H57" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I57" s="20"/>
+      <c r="I57" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J57" s="20" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="K57" s="20" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="L57" s="20">
         <v>6</v>
@@ -4784,14 +4968,18 @@
         <f t="shared" ref="M57" si="49">L57*5</f>
         <v>30</v>
       </c>
-      <c r="N57" s="20"/>
-      <c r="O57" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P57" s="21"/>
+      <c r="N57" s="20">
+        <v>100</v>
+      </c>
+      <c r="O57" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P57" s="21">
+        <v>6.9999999999999999E-4</v>
+      </c>
       <c r="Q57" s="21">
         <f t="shared" ref="Q57" si="50">P57*N57</f>
-        <v>0</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="R57" s="20"/>
     </row>
@@ -4819,12 +5007,14 @@
       <c r="H58" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I58" s="14"/>
+      <c r="I58" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J58" s="14" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="K58" s="14" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="L58" s="14">
         <v>4</v>
@@ -4833,14 +5023,18 @@
         <f>L58*5</f>
         <v>20</v>
       </c>
-      <c r="N58" s="14"/>
-      <c r="O58" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P58" s="15"/>
+      <c r="N58" s="14">
+        <v>100</v>
+      </c>
+      <c r="O58" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P58" s="15">
+        <v>8.9999999999999998E-4</v>
+      </c>
       <c r="Q58" s="15">
         <f>P58*N58</f>
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="R58" s="14"/>
     </row>
@@ -4868,12 +5062,14 @@
       <c r="H59" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I59" s="20"/>
+      <c r="I59" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J59" s="20" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="K59" s="20" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="L59" s="20">
         <v>1</v>
@@ -4882,14 +5078,18 @@
         <f t="shared" ref="M59" si="51">L59*5</f>
         <v>5</v>
       </c>
-      <c r="N59" s="20"/>
-      <c r="O59" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P59" s="21"/>
+      <c r="N59" s="20">
+        <v>100</v>
+      </c>
+      <c r="O59" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P59" s="21">
+        <v>1E-3</v>
+      </c>
       <c r="Q59" s="21">
         <f t="shared" ref="Q59" si="52">P59*N59</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="R59" s="20"/>
     </row>
@@ -4917,12 +5117,14 @@
       <c r="H60" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="I60" s="14"/>
+      <c r="I60" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J60" s="14" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="K60" s="14" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="L60" s="14">
         <v>12</v>
@@ -4931,14 +5133,18 @@
         <f>L60*5</f>
         <v>60</v>
       </c>
-      <c r="N60" s="14"/>
-      <c r="O60" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P60" s="15"/>
+      <c r="N60" s="14">
+        <v>100</v>
+      </c>
+      <c r="O60" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P60" s="15">
+        <v>4.8999999999999998E-3</v>
+      </c>
       <c r="Q60" s="15">
         <f>P60*N60</f>
-        <v>0</v>
+        <v>0.49</v>
       </c>
       <c r="R60" s="14"/>
     </row>
@@ -4966,12 +5172,14 @@
       <c r="H61" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="I61" s="20"/>
+      <c r="I61" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J61" s="20" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="K61" s="20" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L61" s="20">
         <v>1</v>
@@ -4980,14 +5188,18 @@
         <f t="shared" ref="M61" si="53">L61*5</f>
         <v>5</v>
       </c>
-      <c r="N61" s="20"/>
-      <c r="O61" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P61" s="21"/>
+      <c r="N61" s="20">
+        <v>100</v>
+      </c>
+      <c r="O61" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P61" s="21">
+        <v>5.9999999999999995E-4</v>
+      </c>
       <c r="Q61" s="21">
         <f t="shared" ref="Q61" si="54">P61*N61</f>
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="R61" s="20"/>
     </row>
@@ -5015,12 +5227,14 @@
       <c r="H62" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I62" s="14"/>
+      <c r="I62" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J62" s="14" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="K62" s="14" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="L62" s="14">
         <v>1</v>
@@ -5029,14 +5243,18 @@
         <f>L62*5</f>
         <v>5</v>
       </c>
-      <c r="N62" s="14"/>
-      <c r="O62" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P62" s="15"/>
+      <c r="N62" s="14">
+        <v>100</v>
+      </c>
+      <c r="O62" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P62" s="15">
+        <v>6.9999999999999999E-4</v>
+      </c>
       <c r="Q62" s="15">
         <f>P62*N62</f>
-        <v>0</v>
+        <v>6.9999999999999993E-2</v>
       </c>
       <c r="R62" s="14"/>
     </row>
@@ -5049,51 +5267,51 @@
       <c r="C63" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="D63" s="45" t="s">
+      <c r="D63" s="42" t="s">
         <v>86</v>
       </c>
-      <c r="E63" s="45" t="s">
+      <c r="E63" s="42" t="s">
         <v>139</v>
       </c>
-      <c r="F63" s="48" t="s">
+      <c r="F63" s="44" t="s">
         <v>189</v>
       </c>
-      <c r="G63" s="45" t="s">
+      <c r="G63" s="42" t="s">
         <v>237</v>
       </c>
-      <c r="H63" s="45" t="s">
+      <c r="H63" s="42" t="s">
         <v>264</v>
       </c>
-      <c r="I63" s="45" t="s">
-        <v>310</v>
-      </c>
-      <c r="J63" s="45" t="s">
-        <v>333</v>
-      </c>
-      <c r="K63" s="45" t="s">
-        <v>362</v>
-      </c>
-      <c r="L63" s="45">
+      <c r="I63" s="42" t="s">
+        <v>310</v>
+      </c>
+      <c r="J63" s="42" t="s">
+        <v>332</v>
+      </c>
+      <c r="K63" s="42" t="s">
+        <v>361</v>
+      </c>
+      <c r="L63" s="42">
         <v>4</v>
       </c>
-      <c r="M63" s="45">
+      <c r="M63" s="42">
         <f t="shared" ref="M63" si="55">L63*5</f>
         <v>20</v>
       </c>
-      <c r="N63" s="45" t="s">
-        <v>310</v>
-      </c>
-      <c r="O63" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P63" s="50" t="s">
-        <v>310</v>
-      </c>
-      <c r="Q63" s="50" t="s">
-        <v>310</v>
-      </c>
-      <c r="R63" s="51" t="s">
-        <v>405</v>
+      <c r="N63" s="42" t="s">
+        <v>310</v>
+      </c>
+      <c r="O63" s="43" t="s">
+        <v>409</v>
+      </c>
+      <c r="P63" s="46" t="s">
+        <v>310</v>
+      </c>
+      <c r="Q63" s="46" t="s">
+        <v>310</v>
+      </c>
+      <c r="R63" s="47" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="64" spans="1:18" x14ac:dyDescent="0.25">
@@ -5120,12 +5338,14 @@
       <c r="H64" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="I64" s="14"/>
+      <c r="I64" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J64" s="14" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="K64" s="14" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="L64" s="14">
         <v>1</v>
@@ -5134,14 +5354,18 @@
         <f>L64*5</f>
         <v>5</v>
       </c>
-      <c r="N64" s="14"/>
-      <c r="O64" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P64" s="15"/>
+      <c r="N64" s="14">
+        <v>100</v>
+      </c>
+      <c r="O64" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P64" s="15">
+        <v>5.9999999999999995E-4</v>
+      </c>
       <c r="Q64" s="15">
         <f>P64*N64</f>
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="R64" s="14"/>
     </row>
@@ -5161,7 +5385,7 @@
         <v>155</v>
       </c>
       <c r="F65" s="20" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G65" s="20" t="s">
         <v>193</v>
@@ -5169,9 +5393,11 @@
       <c r="H65" s="20" t="s">
         <v>289</v>
       </c>
-      <c r="I65" s="20"/>
+      <c r="I65" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J65" s="20" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="K65" s="20" t="s">
         <v>310</v>
@@ -5183,14 +5409,18 @@
         <f t="shared" ref="M65" si="56">L65*5</f>
         <v>5</v>
       </c>
-      <c r="N65" s="20"/>
-      <c r="O65" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P65" s="21"/>
+      <c r="N65" s="20">
+        <v>10</v>
+      </c>
+      <c r="O65" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P65" s="21">
+        <v>0.1552</v>
+      </c>
       <c r="Q65" s="21">
         <f t="shared" ref="Q65" si="57">P65*N65</f>
-        <v>0</v>
+        <v>1.552</v>
       </c>
       <c r="R65" s="20"/>
     </row>
@@ -5218,9 +5448,11 @@
       <c r="H66" s="14" t="s">
         <v>290</v>
       </c>
-      <c r="I66" s="14"/>
+      <c r="I66" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J66" s="14" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="K66" s="20" t="s">
         <v>310</v>
@@ -5232,14 +5464,18 @@
         <f>L66*5</f>
         <v>5</v>
       </c>
-      <c r="N66" s="14"/>
-      <c r="O66" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P66" s="15"/>
+      <c r="N66" s="14">
+        <v>6</v>
+      </c>
+      <c r="O66" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P66" s="15">
+        <v>2.6966000000000001</v>
+      </c>
       <c r="Q66" s="15">
         <f>P66*N66</f>
-        <v>0</v>
+        <v>16.179600000000001</v>
       </c>
       <c r="R66" s="14"/>
     </row>
@@ -5267,9 +5503,11 @@
       <c r="H67" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="I67" s="20"/>
+      <c r="I67" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J67" s="20" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="K67" s="20" t="s">
         <v>310</v>
@@ -5281,14 +5519,18 @@
         <f t="shared" ref="M67" si="58">L67*5</f>
         <v>5</v>
       </c>
-      <c r="N67" s="20"/>
-      <c r="O67" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P67" s="21"/>
+      <c r="N67" s="20">
+        <v>6</v>
+      </c>
+      <c r="O67" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P67" s="21">
+        <v>0.41870000000000002</v>
+      </c>
       <c r="Q67" s="21">
         <f t="shared" ref="Q67" si="59">P67*N67</f>
-        <v>0</v>
+        <v>2.5122</v>
       </c>
       <c r="R67" s="20"/>
     </row>
@@ -5316,9 +5558,11 @@
       <c r="H68" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="I68" s="14"/>
+      <c r="I68" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J68" s="14" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="K68" s="20" t="s">
         <v>310</v>
@@ -5330,14 +5574,18 @@
         <f>L68*5</f>
         <v>5</v>
       </c>
-      <c r="N68" s="14"/>
-      <c r="O68" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P68" s="15"/>
+      <c r="N68" s="14">
+        <v>10</v>
+      </c>
+      <c r="O68" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P68" s="15">
+        <v>0.1706</v>
+      </c>
       <c r="Q68" s="15">
         <f>P68*N68</f>
-        <v>0</v>
+        <v>1.706</v>
       </c>
       <c r="R68" s="14"/>
     </row>
@@ -5365,9 +5613,11 @@
       <c r="H69" s="20" t="s">
         <v>292</v>
       </c>
-      <c r="I69" s="20"/>
+      <c r="I69" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J69" s="20" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="K69" s="20" t="s">
         <v>310</v>
@@ -5379,14 +5629,18 @@
         <f t="shared" ref="M69" si="60">L69*5</f>
         <v>20</v>
       </c>
-      <c r="N69" s="20"/>
-      <c r="O69" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P69" s="21"/>
+      <c r="N69" s="20">
+        <v>25</v>
+      </c>
+      <c r="O69" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P69" s="21">
+        <v>0.22259999999999999</v>
+      </c>
       <c r="Q69" s="21">
         <f t="shared" ref="Q69" si="61">P69*N69</f>
-        <v>0</v>
+        <v>5.5649999999999995</v>
       </c>
       <c r="R69" s="20"/>
     </row>
@@ -5414,9 +5668,11 @@
       <c r="H70" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="I70" s="14"/>
+      <c r="I70" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J70" s="14" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="K70" s="20" t="s">
         <v>310</v>
@@ -5428,14 +5684,18 @@
         <f>L70*5</f>
         <v>5</v>
       </c>
-      <c r="N70" s="14"/>
-      <c r="O70" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P70" s="15"/>
+      <c r="N70" s="14">
+        <v>6</v>
+      </c>
+      <c r="O70" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P70" s="15">
+        <v>2.9133</v>
+      </c>
       <c r="Q70" s="15">
         <f>P70*N70</f>
-        <v>0</v>
+        <v>17.479800000000001</v>
       </c>
       <c r="R70" s="14"/>
     </row>
@@ -5463,9 +5723,11 @@
       <c r="H71" s="20" t="s">
         <v>293</v>
       </c>
-      <c r="I71" s="20"/>
+      <c r="I71" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J71" s="20" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="K71" s="20" t="s">
         <v>310</v>
@@ -5477,14 +5739,18 @@
         <f t="shared" ref="M71" si="62">L71*5</f>
         <v>5</v>
       </c>
-      <c r="N71" s="20"/>
-      <c r="O71" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P71" s="21"/>
+      <c r="N71" s="20">
+        <v>6</v>
+      </c>
+      <c r="O71" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P71" s="21">
+        <v>0.33610000000000001</v>
+      </c>
       <c r="Q71" s="21">
         <f t="shared" ref="Q71" si="63">P71*N71</f>
-        <v>0</v>
+        <v>2.0165999999999999</v>
       </c>
       <c r="R71" s="20"/>
     </row>
@@ -5512,9 +5778,11 @@
       <c r="H72" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="I72" s="14"/>
+      <c r="I72" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J72" s="14" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="K72" s="20" t="s">
         <v>310</v>
@@ -5526,14 +5794,18 @@
         <f>L72*5</f>
         <v>5</v>
       </c>
-      <c r="N72" s="14"/>
-      <c r="O72" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P72" s="15"/>
+      <c r="N72" s="14">
+        <v>6</v>
+      </c>
+      <c r="O72" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P72" s="15">
+        <v>3.4409999999999998</v>
+      </c>
       <c r="Q72" s="15">
         <f>P72*N72</f>
-        <v>0</v>
+        <v>20.646000000000001</v>
       </c>
       <c r="R72" s="14"/>
     </row>
@@ -5561,9 +5833,11 @@
       <c r="H73" s="20" t="s">
         <v>294</v>
       </c>
-      <c r="I73" s="20"/>
+      <c r="I73" s="14" t="s">
+        <v>310</v>
+      </c>
       <c r="J73" s="20" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="K73" s="20" t="s">
         <v>310</v>
@@ -5575,14 +5849,18 @@
         <f t="shared" ref="M73" si="64">L73*5</f>
         <v>60</v>
       </c>
-      <c r="N73" s="20"/>
-      <c r="O73" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P73" s="21"/>
+      <c r="N73" s="20">
+        <v>65</v>
+      </c>
+      <c r="O73" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P73" s="21">
+        <v>8.8300000000000003E-2</v>
+      </c>
       <c r="Q73" s="21">
         <f t="shared" ref="Q73" si="65">P73*N73</f>
-        <v>0</v>
+        <v>5.7395000000000005</v>
       </c>
       <c r="R73" s="20"/>
     </row>
@@ -5595,51 +5873,51 @@
       <c r="C74" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="D74" s="45" t="s">
+      <c r="D74" s="42" t="s">
         <v>97</v>
       </c>
-      <c r="E74" s="45" t="s">
+      <c r="E74" s="42" t="s">
         <v>164</v>
       </c>
-      <c r="F74" s="46" t="s">
+      <c r="F74" s="43" t="s">
         <v>202</v>
       </c>
-      <c r="G74" s="45" t="s">
+      <c r="G74" s="42" t="s">
         <v>261</v>
       </c>
-      <c r="H74" s="45" t="s">
+      <c r="H74" s="42" t="s">
         <v>295</v>
       </c>
-      <c r="I74" s="45" t="s">
-        <v>310</v>
-      </c>
-      <c r="J74" s="45" t="s">
-        <v>358</v>
-      </c>
-      <c r="K74" s="45" t="s">
-        <v>362</v>
-      </c>
-      <c r="L74" s="45">
+      <c r="I74" s="42" t="s">
+        <v>310</v>
+      </c>
+      <c r="J74" s="42" t="s">
+        <v>357</v>
+      </c>
+      <c r="K74" s="42" t="s">
+        <v>361</v>
+      </c>
+      <c r="L74" s="42">
         <v>1</v>
       </c>
-      <c r="M74" s="45">
+      <c r="M74" s="42">
         <f>L74*5</f>
         <v>5</v>
       </c>
-      <c r="N74" s="45" t="s">
-        <v>310</v>
-      </c>
-      <c r="O74" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P74" s="50" t="s">
-        <v>310</v>
-      </c>
-      <c r="Q74" s="50" t="s">
-        <v>310</v>
-      </c>
-      <c r="R74" s="51" t="s">
-        <v>405</v>
+      <c r="N74" s="42" t="s">
+        <v>310</v>
+      </c>
+      <c r="O74" s="43" t="s">
+        <v>409</v>
+      </c>
+      <c r="P74" s="46" t="s">
+        <v>310</v>
+      </c>
+      <c r="Q74" s="46" t="s">
+        <v>310</v>
+      </c>
+      <c r="R74" s="47" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="75" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5658,7 +5936,7 @@
         <v>165</v>
       </c>
       <c r="F75" s="20" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G75" s="20" t="s">
         <v>262</v>
@@ -5666,12 +5944,14 @@
       <c r="H75" s="20" t="s">
         <v>296</v>
       </c>
-      <c r="I75" s="20"/>
+      <c r="I75" s="20" t="s">
+        <v>310</v>
+      </c>
       <c r="J75" s="20" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="K75" s="20" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="L75" s="20">
         <v>1</v>
@@ -5680,14 +5960,18 @@
         <f t="shared" ref="M75" si="66">L75*5</f>
         <v>5</v>
       </c>
-      <c r="N75" s="20"/>
-      <c r="O75" s="20" t="s">
-        <v>410</v>
-      </c>
-      <c r="P75" s="21"/>
+      <c r="N75" s="20">
+        <v>10</v>
+      </c>
+      <c r="O75" s="49" t="s">
+        <v>409</v>
+      </c>
+      <c r="P75" s="21">
+        <v>0.27510000000000001</v>
+      </c>
       <c r="Q75" s="21">
         <f t="shared" ref="Q75" si="67">P75*N75</f>
-        <v>0</v>
+        <v>2.7510000000000003</v>
       </c>
       <c r="R75" s="20"/>
     </row>
@@ -5705,14 +5989,14 @@
       <c r="K76" s="1"/>
       <c r="L76" s="1"/>
       <c r="M76" s="1"/>
-      <c r="N76" s="43" t="s">
+      <c r="N76" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="O76" s="44"/>
-      <c r="P76" s="44"/>
-      <c r="Q76" s="18" t="e">
-        <f>SUM(#REF!)</f>
-        <v>#REF!</v>
+      <c r="O76" s="52"/>
+      <c r="P76" s="52"/>
+      <c r="Q76" s="18">
+        <f>SUM(Q8:Q75)</f>
+        <v>148.86919999999998</v>
       </c>
       <c r="R76" s="1"/>
     </row>
@@ -5730,14 +6014,14 @@
       <c r="K77" s="1"/>
       <c r="L77" s="1"/>
       <c r="M77" s="1"/>
-      <c r="N77" s="43" t="s">
+      <c r="N77" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="O77" s="44"/>
-      <c r="P77" s="44"/>
-      <c r="Q77" s="19" t="e">
+      <c r="O77" s="52"/>
+      <c r="P77" s="52"/>
+      <c r="Q77" s="19">
         <f>Q76/5</f>
-        <v>#REF!</v>
+        <v>29.773839999999996</v>
       </c>
       <c r="R77" s="1"/>
     </row>
@@ -5775,8 +6059,48 @@
     <hyperlink ref="O31" r:id="rId22"/>
     <hyperlink ref="O33" r:id="rId23"/>
     <hyperlink ref="O34" r:id="rId24"/>
+    <hyperlink ref="O35" r:id="rId25"/>
+    <hyperlink ref="O36" r:id="rId26"/>
+    <hyperlink ref="O37" r:id="rId27"/>
+    <hyperlink ref="O38" r:id="rId28"/>
+    <hyperlink ref="O39" r:id="rId29"/>
+    <hyperlink ref="O40" r:id="rId30"/>
+    <hyperlink ref="O41" r:id="rId31"/>
+    <hyperlink ref="O42" r:id="rId32"/>
+    <hyperlink ref="O43" r:id="rId33"/>
+    <hyperlink ref="O44" r:id="rId34"/>
+    <hyperlink ref="O45" r:id="rId35"/>
+    <hyperlink ref="O47" r:id="rId36"/>
+    <hyperlink ref="O48" r:id="rId37"/>
+    <hyperlink ref="O49" r:id="rId38"/>
+    <hyperlink ref="O50" r:id="rId39"/>
+    <hyperlink ref="O51" r:id="rId40"/>
+    <hyperlink ref="O52" r:id="rId41"/>
+    <hyperlink ref="O53" r:id="rId42"/>
+    <hyperlink ref="O54" r:id="rId43"/>
+    <hyperlink ref="O55" r:id="rId44"/>
+    <hyperlink ref="O56" r:id="rId45"/>
+    <hyperlink ref="O57" r:id="rId46"/>
+    <hyperlink ref="O58" r:id="rId47"/>
+    <hyperlink ref="O59" r:id="rId48"/>
+    <hyperlink ref="O60" r:id="rId49"/>
+    <hyperlink ref="O61" r:id="rId50"/>
+    <hyperlink ref="O62" r:id="rId51"/>
+    <hyperlink ref="O64" r:id="rId52"/>
+    <hyperlink ref="O65" r:id="rId53"/>
+    <hyperlink ref="O66" r:id="rId54"/>
+    <hyperlink ref="O67" r:id="rId55"/>
+    <hyperlink ref="O68" r:id="rId56"/>
+    <hyperlink ref="O69" r:id="rId57"/>
+    <hyperlink ref="O70" r:id="rId58"/>
+    <hyperlink ref="O71" r:id="rId59"/>
+    <hyperlink ref="O72" r:id="rId60"/>
+    <hyperlink ref="O73" r:id="rId61"/>
+    <hyperlink ref="O75" r:id="rId62"/>
+    <hyperlink ref="O32" r:id="rId63"/>
+    <hyperlink ref="O22" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId25"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId65"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#29 Client and eSpark BOM added
</commit_message>
<xml_diff>
--- a/Design Files/BLDC-Board-v1.0/BOM/eSpark_BOM_BLDC-Board-v1.0.xlsx
+++ b/Design Files/BLDC-Board-v1.0/BOM/eSpark_BOM_BLDC-Board-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="715" uniqueCount="414">
   <si>
     <t>Component list</t>
   </si>
@@ -1261,9 +1261,6 @@
   </si>
   <si>
     <t>C49257</t>
-  </si>
-  <si>
-    <t>C2688120</t>
   </si>
 </sst>
 </file>
@@ -3031,9 +3028,7 @@
       <c r="I22" s="20" t="s">
         <v>310</v>
       </c>
-      <c r="J22" s="14" t="s">
-        <v>414</v>
-      </c>
+      <c r="J22" s="14"/>
       <c r="K22" s="20" t="s">
         <v>310</v>
       </c>
@@ -3047,15 +3042,11 @@
       <c r="N22" s="14">
         <v>20</v>
       </c>
-      <c r="O22" s="49" t="s">
-        <v>409</v>
-      </c>
-      <c r="P22" s="15">
-        <v>3.3500000000000002E-2</v>
-      </c>
+      <c r="O22" s="49"/>
+      <c r="P22" s="15"/>
       <c r="Q22" s="15">
         <f>P22*N22</f>
-        <v>0.67</v>
+        <v>0</v>
       </c>
       <c r="R22" s="14"/>
     </row>
@@ -5996,7 +5987,7 @@
       <c r="P76" s="52"/>
       <c r="Q76" s="18">
         <f>SUM(Q8:Q75)</f>
-        <v>148.86919999999998</v>
+        <v>148.19919999999999</v>
       </c>
       <c r="R76" s="1"/>
     </row>
@@ -6021,7 +6012,7 @@
       <c r="P77" s="52"/>
       <c r="Q77" s="19">
         <f>Q76/5</f>
-        <v>29.773839999999996</v>
+        <v>29.63984</v>
       </c>
       <c r="R77" s="1"/>
     </row>
@@ -6098,9 +6089,8 @@
     <hyperlink ref="O73" r:id="rId61"/>
     <hyperlink ref="O75" r:id="rId62"/>
     <hyperlink ref="O32" r:id="rId63"/>
-    <hyperlink ref="O22" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId65"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId64"/>
 </worksheet>
 </file>
</xml_diff>